<commit_message>
limpieza redacción en código
</commit_message>
<xml_diff>
--- a/docs/Matriz_Infraestructura.xlsx
+++ b/docs/Matriz_Infraestructura.xlsx
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TrazaDoc — MVP de verificación de integridad y trazabilidad documental en contratos laborales con blockchain permisionada (Hyperledger Fabric)</t>
+          <t>TrazaDoc: MVP de verificación de integridad y trazabilidad documental en contratos laborales con blockchain permisionada (Hyperledger Fabric)</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Objetivo específico: OE2 — Diseñar la arquitectura del sistema (UX/UI, software e infraestructura sobre Hyperledger Fabric desplegada en Docker).</t>
+          <t>Objetivo específico: OE2, Diseñar la arquitectura del sistema (UX/UI, software e infraestructura sobre Hyperledger Fabric desplegada en Docker).</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Autoras: Laura Sofia Diaz Suarez · Sofia Ortiz Daza — Universidad Católica de Colombia</t>
+          <t>Autoras: Laura Sofia Diaz Suarez · Sofia Ortiz Daza, Universidad Católica de Colombia</t>
         </is>
       </c>
     </row>
@@ -554,56 +554,56 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>1. Componentes — cada nodo/servicio: tecnología, versión, función, puertos, persistencia, seguridad, dependencias y requisitos que cumple.</t>
+          <t>1. Componentes: cada nodo/servicio: tecnología, versión, función, puertos, persistencia, seguridad, dependencias y requisitos que cumple.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2. Red Fabric — topología blockchain: organizaciones, canal, consenso, políticas, chaincode.</t>
+          <t>2. Red Fabric: topología blockchain: organizaciones, canal, consenso, políticas, chaincode.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>3. Puertos — mapa de puertos expuestos en el host.</t>
+          <t>3. Puertos: mapa de puertos expuestos en el host.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>4. Configuración — variables de entorno y secretos.</t>
+          <t>4. Configuración: variables de entorno y secretos.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>5. Despliegue — procedimiento reproducible paso a paso.</t>
+          <t>5. Despliegue: procedimiento reproducible paso a paso.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>6. Trazabilidad RNF — qué componente cumple cada requisito no funcional de infraestructura.</t>
+          <t>6. Trazabilidad RNF: qué componente cumple cada requisito no funcional de infraestructura.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>7. Observaciones — decisiones de diseño y diferencias entre lo documentado y lo implementado.</t>
+          <t>7. Observaciones: decisiones de diseño y diferencias entre lo documentado y lo implementado.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>8. Aprobación — registro de revisión del tutor (KPI OE2).</t>
+          <t>8. Aprobación: registro de revisión del tutor (KPI OE2).</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>— (solo lo invoca el peer)</t>
+          <t>: (solo lo invoca el peer)</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1413,12 +1413,12 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1480,17 +1480,17 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>— (servicio en la nube)</t>
+          <t>: (servicio en la nube)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Plan de Sprint 0 (D2) y Sprint 2 (D7): OR('Org1MSP.peer','Org2MSP.peer') — basta una organización.</t>
+          <t>Plan de Sprint 0 (D2) y Sprint 2 (D7): OR('Org1MSP.peer','Org2MSP.peer'), basta una organización.</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">

</xml_diff>